<commit_message>
Termine de contruiur la base
</commit_message>
<xml_diff>
--- a/Datos/Crudos/agbarometerUSA_marzo2026.xlsx
+++ b/Datos/Crudos/agbarometerUSA_marzo2026.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smithse/CCA_Purdue Dropbox/CCA_Purdue Team Folder/1. Purdue-CME Ag Barometer/7. Website/Table pdfs/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Facultad\Practica Profesional\Practica-Profesional-Privado\Datos\Crudos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A2D8240-733B-0B47-8AF2-B47957110713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="4100"/>
   </bookViews>
   <sheets>
     <sheet name="AgEconomyBarometer_SurveryHisto" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,10 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="17">
-  <si>
-    <t>Month/Year</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="18">
   <si>
     <t>Purdue/CME Ag Economy Barometer</t>
   </si>
@@ -85,11 +81,17 @@
   <si>
     <t>September</t>
   </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -601,48 +603,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -953,9 +955,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F127"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -963,27 +965,29 @@
     <col min="4" max="6" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
       </c>
       <c r="B2">
         <v>2015</v>
@@ -1001,9 +1005,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>2015</v>
@@ -1021,9 +1025,9 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>2015</v>
@@ -1041,9 +1045,9 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>2016</v>
@@ -1061,9 +1065,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>2016</v>
@@ -1081,9 +1085,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>2016</v>
@@ -1101,9 +1105,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>2016</v>
@@ -1121,9 +1125,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>2016</v>
@@ -1141,9 +1145,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>2016</v>
@@ -1161,9 +1165,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>2016</v>
@@ -1181,9 +1185,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>2016</v>
@@ -1201,9 +1205,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>2016</v>
@@ -1221,9 +1225,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14">
         <v>2016</v>
@@ -1241,9 +1245,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15">
         <v>2016</v>
@@ -1261,9 +1265,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16">
         <v>2016</v>
@@ -1281,9 +1285,9 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17">
         <v>2017</v>
@@ -1301,9 +1305,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18">
         <v>2017</v>
@@ -1321,9 +1325,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>2017</v>
@@ -1341,9 +1345,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20">
         <v>2017</v>
@@ -1361,9 +1365,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21">
         <v>2017</v>
@@ -1381,9 +1385,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22">
         <v>2017</v>
@@ -1401,9 +1405,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B23">
         <v>2017</v>
@@ -1421,9 +1425,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24">
         <v>2017</v>
@@ -1441,9 +1445,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B25">
         <v>2017</v>
@@ -1461,9 +1465,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26">
         <v>2017</v>
@@ -1481,9 +1485,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27">
         <v>2017</v>
@@ -1501,9 +1505,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B28">
         <v>2017</v>
@@ -1521,9 +1525,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29">
         <v>2018</v>
@@ -1541,9 +1545,9 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B30">
         <v>2018</v>
@@ -1561,9 +1565,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B31">
         <v>2018</v>
@@ -1581,9 +1585,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B32">
         <v>2018</v>
@@ -1601,9 +1605,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33">
         <v>2018</v>
@@ -1621,9 +1625,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34">
         <v>2018</v>
@@ -1641,9 +1645,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B35">
         <v>2018</v>
@@ -1661,9 +1665,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B36">
         <v>2018</v>
@@ -1681,9 +1685,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B37">
         <v>2018</v>
@@ -1701,9 +1705,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38">
         <v>2018</v>
@@ -1721,9 +1725,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B39">
         <v>2018</v>
@@ -1741,9 +1745,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40">
         <v>2018</v>
@@ -1761,9 +1765,9 @@
         <v>51</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41">
         <v>2019</v>
@@ -1781,9 +1785,9 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B42">
         <v>2019</v>
@@ -1801,9 +1805,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B43">
         <v>2019</v>
@@ -1821,9 +1825,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B44">
         <v>2019</v>
@@ -1841,9 +1845,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B45">
         <v>2019</v>
@@ -1861,9 +1865,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46">
         <v>2019</v>
@@ -1881,9 +1885,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47">
         <v>2019</v>
@@ -1901,9 +1905,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48">
         <v>2019</v>
@@ -1921,9 +1925,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B49">
         <v>2019</v>
@@ -1941,9 +1945,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B50">
         <v>2019</v>
@@ -1961,9 +1965,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B51">
         <v>2019</v>
@@ -1981,9 +1985,9 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B52">
         <v>2019</v>
@@ -2001,9 +2005,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B53">
         <v>2020</v>
@@ -2021,9 +2025,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B54">
         <v>2020</v>
@@ -2041,9 +2045,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B55">
         <v>2020</v>
@@ -2061,9 +2065,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B56">
         <v>2020</v>
@@ -2081,9 +2085,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B57">
         <v>2020</v>
@@ -2101,9 +2105,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B58">
         <v>2020</v>
@@ -2121,9 +2125,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B59">
         <v>2020</v>
@@ -2141,9 +2145,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B60">
         <v>2020</v>
@@ -2161,9 +2165,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B61">
         <v>2020</v>
@@ -2181,9 +2185,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B62">
         <v>2020</v>
@@ -2201,9 +2205,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B63">
         <v>2020</v>
@@ -2221,9 +2225,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B64">
         <v>2020</v>
@@ -2241,9 +2245,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B65">
         <v>2021</v>
@@ -2261,9 +2265,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B66">
         <v>2021</v>
@@ -2281,9 +2285,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B67">
         <v>2021</v>
@@ -2301,9 +2305,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68">
         <v>2021</v>
@@ -2321,9 +2325,9 @@
         <v>75</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69">
         <v>2021</v>
@@ -2341,9 +2345,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B70">
         <v>2021</v>
@@ -2361,9 +2365,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B71">
         <v>2021</v>
@@ -2381,9 +2385,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B72">
         <v>2021</v>
@@ -2401,9 +2405,9 @@
         <v>53</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B73">
         <v>2021</v>
@@ -2421,9 +2425,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B74">
         <v>2021</v>
@@ -2441,9 +2445,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B75">
         <v>2021</v>
@@ -2461,9 +2465,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B76">
         <v>2021</v>
@@ -2481,9 +2485,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B77">
         <v>2022</v>
@@ -2501,9 +2505,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B78">
         <v>2022</v>
@@ -2521,9 +2525,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B79">
         <v>2022</v>
@@ -2541,9 +2545,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B80">
         <v>2022</v>
@@ -2561,9 +2565,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B81">
         <v>2022</v>
@@ -2581,9 +2585,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B82">
         <v>2022</v>
@@ -2601,9 +2605,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B83">
         <v>2022</v>
@@ -2621,9 +2625,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B84">
         <v>2022</v>
@@ -2641,9 +2645,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B85">
         <v>2022</v>
@@ -2661,9 +2665,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B86">
         <v>2022</v>
@@ -2681,9 +2685,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B87">
         <v>2022</v>
@@ -2701,9 +2705,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B88">
         <v>2022</v>
@@ -2721,9 +2725,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B89">
         <v>2023</v>
@@ -2741,9 +2745,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B90">
         <v>2023</v>
@@ -2761,9 +2765,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B91">
         <v>2023</v>
@@ -2781,9 +2785,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B92">
         <v>2023</v>
@@ -2801,9 +2805,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B93">
         <v>2023</v>
@@ -2821,9 +2825,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B94">
         <v>2023</v>
@@ -2841,9 +2845,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B95">
         <v>2023</v>
@@ -2861,9 +2865,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B96">
         <v>2023</v>
@@ -2881,9 +2885,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B97">
         <v>2023</v>
@@ -2901,9 +2905,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B98">
         <v>2023</v>
@@ -2921,9 +2925,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B99">
         <v>2023</v>
@@ -2941,9 +2945,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B100">
         <v>2023</v>
@@ -2961,9 +2965,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B101">
         <v>2024</v>
@@ -2981,9 +2985,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B102">
         <v>2024</v>
@@ -3001,9 +3005,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B103">
         <v>2024</v>
@@ -3021,9 +3025,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B104">
         <v>2024</v>
@@ -3041,9 +3045,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B105">
         <v>2024</v>
@@ -3061,9 +3065,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B106">
         <v>2024</v>
@@ -3081,9 +3085,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B107">
         <v>2024</v>
@@ -3101,9 +3105,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B108">
         <v>2024</v>
@@ -3121,9 +3125,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B109">
         <v>2024</v>
@@ -3141,9 +3145,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B110">
         <v>2024</v>
@@ -3161,9 +3165,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B111">
         <v>2024</v>
@@ -3181,9 +3185,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B112">
         <v>2024</v>
@@ -3201,9 +3205,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B113">
         <v>2025</v>
@@ -3221,9 +3225,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B114">
         <v>2025</v>
@@ -3241,9 +3245,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B115">
         <v>2025</v>
@@ -3261,9 +3265,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B116">
         <v>2025</v>
@@ -3281,9 +3285,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B117">
         <v>2025</v>
@@ -3301,9 +3305,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B118">
         <v>2025</v>
@@ -3321,9 +3325,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B119">
         <v>2025</v>
@@ -3341,9 +3345,9 @@
         <v>53</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B120">
         <v>2025</v>
@@ -3361,9 +3365,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B121">
         <v>2025</v>
@@ -3381,9 +3385,9 @@
         <v>53</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B122">
         <v>2025</v>
@@ -3401,9 +3405,9 @@
         <v>62</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B123">
         <v>2025</v>
@@ -3421,9 +3425,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B124">
         <v>2025</v>
@@ -3441,9 +3445,9 @@
         <v>58</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B125">
         <v>2026</v>
@@ -3461,9 +3465,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B126">
         <v>2026</v>
@@ -3481,9 +3485,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B127">
         <v>2026</v>

</xml_diff>